<commit_message>
Payer label: 'Payer not stated in the paper'; the who-bears-the-cost table lists a repeated figure once
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/downloads/1BKCLntBLcvoY64pRzy6UIEZ.xlsx
+++ b/data/downloads/1BKCLntBLcvoY64pRzy6UIEZ.xlsx
@@ -845,7 +845,7 @@
       </c>
       <c r="M2" s="1" t="inlineStr">
         <is>
-          <t>Payer unclear</t>
+          <t>Payer not stated in the paper</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
       </c>
       <c r="M3" s="1" t="inlineStr">
         <is>
-          <t>Payer unclear</t>
+          <t>Payer not stated in the paper</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="M4" s="1" t="inlineStr">
         <is>
-          <t>Payer unclear</t>
+          <t>Payer not stated in the paper</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="M5" s="1" t="inlineStr">
         <is>
-          <t>Payer unclear</t>
+          <t>Payer not stated in the paper</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>Payer unclear</t>
+          <t>Payer not stated in the paper</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>Payer unclear</t>
+          <t>Payer not stated in the paper</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>Payer unclear</t>
+          <t>Payer not stated in the paper</t>
         </is>
       </c>
     </row>

</xml_diff>